<commit_message>
Fix truncated control text in CCC-1:2020 (heal page-break splits)
Descriptions were truncated where the official PDF glued page-break banners onto
the end of content lines, and where words were split by hyphenated line-breaks.
Reworked the extractor to strip banners while preserving trailing text and to
heal hyphenated breaks. All 55 controls now carry complete normative text.
Addresses CodeRabbit review feedback.
</commit_message>
<xml_diff>
--- a/tools/excel/ccc/ccc-1-2020.xlsx
+++ b/tools/excel/ccc/ccc-1-2020.xlsx
@@ -995,7 +995,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Cybersecurity risk management methodology mentioned in the ECC Subdomain 1-5 shall also include for the CST, as a minimum: (1) Defining acceptable risk levels for the cloud services. (2) Considering data and information classification accredited by CST in cybersecurity risk management methodology. (3) Developing cybersecurity risk register for cloud services, and monitoring it</t>
+          <t>Cybersecurity risk management methodology mentioned in the ECC Subdomain 1-5 shall also include for the CST, as a minimum: (1) Defining acceptable risk levels for the cloud services. (2) Considering data and information classification accredited by CST in cybersecurity risk management methodology. (3) Developing cybersecurity risk register for cloud services, and monitoring it periodically according to the risks.</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Cybersecurity requirements for change management within the CSP shall be applied and</t>
+          <t>Cybersecurity requirements for change management within the CSP shall be applied and reviewed periodically.</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>In addition to subcontrols in the ECC control 2-2-3, the CST shall cover the following additional subcontrols for cybersecurity requirements for identity and access management requirements, as a minimum: (1) Identity and access management for all cloud credentials along their full lifecycle. (2) Confidentiality of cloud user identification, cloud credential and cloud access rights information, including the requirement on users to keep them private (for employed, third party and CST personnel). (3) Secure session management, including session authenticity, session lockout, and session timeout termination on the cloud. (4) Multi-factor authentication for privileged cloud users. (5) Formal process to detect and prevent unauthorized access to cloud (such as</t>
+          <t>In addition to subcontrols in the ECC control 2-2-3, the CST shall cover the following additional subcontrols for cybersecurity requirements for identity and access management requirements, as a minimum: (1) Identity and access management for all cloud credentials along their full lifecycle. (2) Confidentiality of cloud user identification, cloud credential and cloud access rights information, including the requirement on users to keep them private (for employed, third party and CST personnel). (3) Secure session management, including session authenticity, session lockout, and session timeout termination on the cloud. (4) Multi-factor authentication for privileged cloud users. (5) Formal process to detect and prevent unauthorized access to cloud (such as a threshold of unsuccessful login attempts).</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>In addition to subcontrols in the ECC control 2-3-3, the CSP shall cover the following additional subcontrols for cybersecurity requirements for information system and processing facilities protection requirements, as a minimum: (1) Ensuring that all configurations are applied in accordance to CSP’s cybersecurity standards. (2) Assurance of separation and isolation of data, environments and information systems across CSTs, to prevent data commingling. (3) Adopting of cybersecurity principles for technical system configurations adhering to the minimum functionality principle. (4) Ability of the Cloud Technology Stacks to securely handle input validation, exceptions and failure. (5) Full isolation of security functions and applications from other functions and applications in the Cloud Technology Stack. (6) Notification to CSTs with cybersecurity requirements provided by the CSP that are useable by the CST. (7) Detection and prevention of unauthorized changes to softwares, and systems. (8) Complete isolation and protection of multiple guest environments. (9) The community cloud services provided to CSTs (government organizations and CNI organizations) shall be isolated from any other cloud computing provided to organizations outside the scope of work. (10) Provide cloud computing services from within the KSA, including systems used for storage, processing, and disaster recovery centers. (11) Provide cloud computing services from within the KSA, including systems used for monitoring, and support. (12) Modern technologies, such as Endpoint Detection and Response (EDR) technologies, to ensure that the information servers and devices of CSP’s information processing systems and devices of are ready for rapid response</t>
+          <t>In addition to subcontrols in the ECC control 2-3-3, the CSP shall cover the following additional subcontrols for cybersecurity requirements for information system and processing facilities protection requirements, as a minimum: (1) Ensuring that all configurations are applied in accordance to CSP’s cybersecurity standards. (2) Assurance of separation and isolation of data, environments and information systems across CSTs, to prevent data commingling. (3) Adopting of cybersecurity principles for technical system configurations adhering to the minimum functionality principle. (4) Ability of the Cloud Technology Stacks to securely handle input validation, exceptions and failure. (5) Full isolation of security functions and applications from other functions and applications in the Cloud Technology Stack. (6) Notification to CSTs with cybersecurity requirements provided by the CSP that are useable by the CST. (7) Detection and prevention of unauthorized changes to softwares, and systems. (8) Complete isolation and protection of multiple guest environments. (9) The community cloud services provided to CSTs (government organizations and CNI organizations) shall be isolated from any other cloud computing provided to organizations outside the scope of work. (10) Provide cloud computing services from within the KSA, including systems used for storage, processing, and disaster recovery centers. (11) Provide cloud computing services from within the KSA, including systems used for monitoring, and support. (12) Modern technologies, such as Endpoint Detection and Response (EDR) technologies, to ensure that the information servers and devices of CSP’s information processing systems and devices of are ready for rapid response to incidents.</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>In addition to subcontrols in the ECC control 2-7-3, the CST shall cover the following additional subcontrols for cybersecurity requirements for protecting CST’s data and infor - (1) Exit Strategy to ensure means for secure disposal of data on termination or expiry of the contract with the CSP. (2) Using secure means to export and transfer data and virtual infrastructure.</t>
+          <t>In addition to subcontrols in the ECC control 2-7-3, the CST shall cover the following additional subcontrols for cybersecurity requirements for protecting CST’s data and information in cloud computing, as a minimum: (1) Exit Strategy to ensure means for secure disposal of data on termination or expiry of the contract with the CSP. (2) Using secure means to export and transfer data and virtual infrastructure.</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>In addition to subcontrols in the ECC control 2-9-3, the CSP shall cover the following additional subcontrols for cybersecurity requirements for backup and recovery management, as a minimum: (1) Securing access, storage and transfer of CST’s data backups and its mediums, and protecting it against damage, amendment or unauthorized access. (2) Securing access, storage and transfer of Cloud Technology Stack backups and its mediums, and protecting it against damage, amendment or unau -</t>
+          <t>In addition to subcontrols in the ECC control 2-9-3, the CSP shall cover the following additional subcontrols for cybersecurity requirements for backup and recovery management, as a minimum: (1) Securing access, storage and transfer of CST’s data backups and its mediums, and protecting it against damage, amendment or unauthorized access. (2) Securing access, storage and transfer of Cloud Technology Stack backups and its mediums, and protecting it against damage, amendment or unauthorized access.</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>In addition to subcontrols in the ECC control 2-13-3, the CSP shall cover the following additional subcontrols for cybersecurity requirements for cybersecurity incident and threat (1) Subscribing in authorized and specialized organizations and groups to stay up-to-date on cybersecurity threats, common practices and key know-how. (2) Training for employees and third-party personnel to respond to cybersecurity incidents, in line with their roles and responsibilities. (3) Periodically testing the incident response capability. (4) Root Cause Analysis of cybersecurity incidents and developing plans to address them. (5) Support the CST in cases legal proceedings and forensics, protecting the chain of custody that falls under the management and responsibility of the CSP, in accordance with the related law and regulatory requirements. (6) Real-time reporting to the CST of incidents that may affect CST; if the incident is discovered. (7) Support for CSTs to handle security incidents according to the agreement between the CSP and CST. (8) Measuring and monitoring cybersecurity incident metrics and monitor compliance with contracts and legislative requirements</t>
+          <t>In addition to subcontrols in the ECC control 2-13-3, the CSP shall cover the following additional subcontrols for cybersecurity requirements for cybersecurity incident and threat management, as a minimum: (1) Subscribing in authorized and specialized organizations and groups to stay up-to-date on cybersecurity threats, common practices and key know-how. (2) Training for employees and third-party personnel to respond to cybersecurity incidents, in line with their roles and responsibilities. (3) Periodically testing the incident response capability. (4) Root Cause Analysis of cybersecurity incidents and developing plans to address them. (5) Support the CST in cases legal proceedings and forensics, protecting the chain of custody that falls under the management and responsibility of the CSP, in accordance with the related law and regulatory requirements. (6) Real-time reporting to the CST of incidents that may affect CST; if the incident is discovered. (7) Support for CSTs to handle security incidents according to the agreement between the CSP and CST. (8) Measuring and monitoring cybersecurity incident metrics and monitor compliance with contracts and legislative requirements</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>In addition to subcontrols in the ECC control 2-15-3, the CSP shall cover the following additional subcontrols for cybersecurity requirements for web application security, as a (1) Protecting information involved in application service transactions against possible risks (e.g.: incomplete transmission, mis-routing, unauthorized message alteration, unauthorized disclosure….).</t>
+          <t>In addition to subcontrols in the ECC control 2-15-3, the CSP shall cover the following additional subcontrols for cybersecurity requirements for web application security, as a minimum: (1) Protecting information involved in application service transactions against possible risks (e.g.: incomplete transmission, mis-routing, unauthorized message alteration, unauthorized disclosure….).</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Cybersecurity requirements for usage of information and data media within the CSP shall</t>
+          <t>Cybersecurity requirements for usage of information and data media within the CSP shall be applied and reviewed periodically.</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>In addition to implementing the ECC controls 4-1-2 and 4-1-3, the CSP shall cover the following additional subcontrols for third-party cybersecurity requirements, as a minimum: (1) Ensure that the CSP fulfills NCA's requests to remove software or services, provided by third-party providers that may be considered a cybersecurity threat to national organizations, from the marketplace provided to CSTs. (2) Requirement to provide security documentation for any equipment or services from suppliers and third-party providers. (3) Third party providers compliant with law and regulatory requirements relevant to their scope. (4) Risk management and security governance on third-party providers as part of general cybersecurity risk management and governance. Annex No. (A): Cloud Cybersecurity Controls Levels Cybersecurity controls for cloud services are divided into four levels using a top down approach, level 1, level 2, level 3, and level 4: • Level 1: A classification level applies to data classified as a (top secret) based on what is issued by the competent authority. • Level 2: A classification level applies to data classified as a (secret) based on what is issued by the competent authority. • Level 3: A classification level applies to data classified as a (confidential) based on what is issued by the competent authority. • Level 4: classification level applies to data classified as a (public) based on what is issued by the competent authority. Please note that the highest level of classification should be adopted when the content of an integrated set</t>
+          <t>In addition to implementing the ECC controls 4-1-2 and 4-1-3, the CSP shall cover the following additional subcontrols for third-party cybersecurity requirements, as a minimum: (1) Ensure that the CSP fulfills NCA's requests to remove software or services, provided by third-party providers that may be considered a cybersecurity threat to national organizations, from the marketplace provided to CSTs. (2) Requirement to provide security documentation for any equipment or services from suppliers and third-party providers. (3) Third party providers compliant with law and regulatory requirements relevant to their scope. (4) Risk management and security governance on third-party providers as part of general cybersecurity risk management and governance. Annex No. (A): Cloud Cybersecurity Controls Levels Cybersecurity controls for cloud services are divided into four levels using a top down approach, level 1, level 2, level 3, and level 4: • Level 1: A classification level applies to data classified as a (top secret) based on what is issued by the competent authority. • Level 2: A classification level applies to data classified as a (secret) based on what is issued by the competent authority. • Level 3: A classification level applies to data classified as a (confidential) based on what is issued by the competent authority. • Level 4: classification level applies to data classified as a (public) based on what is issued by the competent authority. Please note that the highest level of classification should be adopted when the content of an integrated set of data includes different levels.</t>
         </is>
       </c>
     </row>

</xml_diff>